<commit_message>
Update July 7 applicants count
</commit_message>
<xml_diff>
--- a/DATA/manual-dashboard-data.xlsx
+++ b/DATA/manual-dashboard-data.xlsx
@@ -158,7 +158,7 @@
         <v>241</v>
       </c>
       <c r="P3">
-        <v>100</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4">
@@ -217,7 +217,7 @@
         <v>241</v>
       </c>
       <c r="P5">
-        <v>100</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update current applicants chart series
</commit_message>
<xml_diff>
--- a/DATA/manual-dashboard-data.xlsx
+++ b/DATA/manual-dashboard-data.xlsx
@@ -14,7 +14,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:Q5"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="32" width="18" customWidth="1"/>
@@ -101,6 +101,11 @@
           <t>07.07.2026</t>
         </is>
       </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>08.07.2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -158,7 +163,10 @@
         <v>241</v>
       </c>
       <c r="P3">
-        <v>197</v>
+        <v>194</v>
+      </c>
+      <c r="Q3">
+        <v>129</v>
       </c>
     </row>
     <row r="4">
@@ -217,7 +225,10 @@
         <v>241</v>
       </c>
       <c r="P5">
-        <v>197</v>
+        <v>194</v>
+      </c>
+      <c r="Q5">
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update admissions data and KCP progress
</commit_message>
<xml_diff>
--- a/DATA/manual-dashboard-data.xlsx
+++ b/DATA/manual-dashboard-data.xlsx
@@ -14,7 +14,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:W5"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="32" width="18" customWidth="1"/>
@@ -106,6 +106,36 @@
           <t>08.07.2026</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>09.07.2026</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>10.07.2026</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>11.07.2026</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>13.07.2026</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>14.07.2026</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>15.07.2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -168,6 +198,24 @@
       <c r="Q3">
         <v>129</v>
       </c>
+      <c r="R3">
+        <v>169</v>
+      </c>
+      <c r="S3">
+        <v>153</v>
+      </c>
+      <c r="T3">
+        <v>111</v>
+      </c>
+      <c r="U3">
+        <v>237</v>
+      </c>
+      <c r="V3">
+        <v>218</v>
+      </c>
+      <c r="W3">
+        <v>221</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -229,6 +277,24 @@
       </c>
       <c r="Q5">
         <v>129</v>
+      </c>
+      <c r="R5">
+        <v>169</v>
+      </c>
+      <c r="S5">
+        <v>153</v>
+      </c>
+      <c r="T5">
+        <v>111</v>
+      </c>
+      <c r="U5">
+        <v>237</v>
+      </c>
+      <c r="V5">
+        <v>218</v>
+      </c>
+      <c r="W5">
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -677,7 +743,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>8575</v>
+        <v>13201</v>
       </c>
     </row>
     <row r="3">
@@ -687,7 +753,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>1526</v>
+        <v>2414</v>
       </c>
     </row>
   </sheetData>
@@ -721,7 +787,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>1526</v>
+        <v>2414</v>
       </c>
     </row>
     <row r="3">
@@ -731,7 +797,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>7049</v>
+        <v>10787</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update admissions data for July 20
</commit_message>
<xml_diff>
--- a/DATA/manual-dashboard-data.xlsx
+++ b/DATA/manual-dashboard-data.xlsx
@@ -14,7 +14,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W5"/>
+  <dimension ref="A1:AA5"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="32" width="18" customWidth="1"/>
@@ -136,6 +136,26 @@
           <t>15.07.2026</t>
         </is>
       </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>16.07.2026</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>17.07.2026</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>18.07.2026</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>20.07.2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -216,6 +236,18 @@
       <c r="W3">
         <v>221</v>
       </c>
+      <c r="X3">
+        <v>205</v>
+      </c>
+      <c r="Y3">
+        <v>198</v>
+      </c>
+      <c r="Z3">
+        <v>95</v>
+      </c>
+      <c r="AA3">
+        <v>367</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -295,6 +327,18 @@
       </c>
       <c r="W5">
         <v>221</v>
+      </c>
+      <c r="X5">
+        <v>205</v>
+      </c>
+      <c r="Y5">
+        <v>198</v>
+      </c>
+      <c r="Z5">
+        <v>95</v>
+      </c>
+      <c r="AA5">
+        <v>367</v>
       </c>
     </row>
   </sheetData>
@@ -743,7 +787,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>13201</v>
+        <v>15791</v>
       </c>
     </row>
     <row r="3">
@@ -753,7 +797,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>2414</v>
+        <v>3021</v>
       </c>
     </row>
   </sheetData>
@@ -787,7 +831,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>2414</v>
+        <v>3021</v>
       </c>
     </row>
     <row r="3">
@@ -797,7 +841,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>10787</v>
+        <v>12770</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update admissions data for August 17
</commit_message>
<xml_diff>
--- a/DATA/manual-dashboard-data.xlsx
+++ b/DATA/manual-dashboard-data.xlsx
@@ -14,7 +14,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK5"/>
+  <dimension ref="A1:AP5"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
     <col min="2" max="32" width="18" customWidth="1"/>
@@ -206,6 +206,31 @@
           <t>07.08.2026</t>
         </is>
       </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>10.08.2026</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>11.08.2026</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>12.08.2026</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>13.08.2026</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>14.08.2026</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -326,7 +351,22 @@
         <v>8</v>
       </c>
       <c r="AK3">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="AL3">
+        <v>80</v>
+      </c>
+      <c r="AM3">
+        <v>35</v>
+      </c>
+      <c r="AN3">
+        <v>33</v>
+      </c>
+      <c r="AO3">
+        <v>27</v>
+      </c>
+      <c r="AP3">
+        <v>30</v>
       </c>
     </row>
     <row r="4">
@@ -448,7 +488,22 @@
         <v>8</v>
       </c>
       <c r="AK5">
-        <v>0</v>
+        <v>11</v>
+      </c>
+      <c r="AL5">
+        <v>80</v>
+      </c>
+      <c r="AM5">
+        <v>35</v>
+      </c>
+      <c r="AN5">
+        <v>33</v>
+      </c>
+      <c r="AO5">
+        <v>27</v>
+      </c>
+      <c r="AP5">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -897,7 +952,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>16767</v>
+        <v>17856</v>
       </c>
     </row>
     <row r="3">
@@ -907,7 +962,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>3629</v>
+        <v>3901</v>
       </c>
     </row>
   </sheetData>
@@ -941,7 +996,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>3629</v>
+        <v>3901</v>
       </c>
     </row>
     <row r="3">
@@ -951,7 +1006,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>13138</v>
+        <v>13955</v>
       </c>
     </row>
   </sheetData>

</xml_diff>